<commit_message>
update example with original value 35a7660f84359ef6af5a985226c0bec9bff7aa5f
</commit_message>
<xml_diff>
--- a/nr-add-lipids/ig/StructureDefinition-mesures-observation-glucose.xlsx
+++ b/nr-add-lipids/ig/StructureDefinition-mesures-observation-glucose.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-01-19T08:51:58+00:00</t>
+    <t>2026-01-19T09:23:14+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -683,7 +683,7 @@
 </t>
   </si>
   <si>
-    <t>Origine de la donnée</t>
+    <t>Valeur d'origine de la donnée. Cette extension est présente uniquement si le résultat contenu dans Observation.value provient d'une conversion (par ex. g/L converti en mmol/L)</t>
   </si>
   <si>
     <t>Extension pour tracer l'origine de la donnée issue d'un compte rendu de biologie (CR-Bio).</t>

</xml_diff>